<commit_message>
added button to start move,changed location names
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel sheets/LocationData.xlsx
+++ b/Assets/Resources/Excel sheets/LocationData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Scratch\s3841792\VANDERBILT\Assets\Resources\Excel sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artem\Desktop\RMIT\RMIT sem 2 2026\GDS6\VANDERBILT\Assets\Resources\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8EA92B8-E058-4437-96A0-0FC11622D980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF27505-049A-461E-A061-B7A1D4779C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="3135" windowWidth="28800" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Faction</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>LocationType</t>
   </si>
@@ -42,21 +36,12 @@
     <t>Mine</t>
   </si>
   <si>
-    <t>Market</t>
-  </si>
-  <si>
-    <t>Warehouse</t>
-  </si>
-  <si>
     <t>Residential</t>
   </si>
   <si>
     <t>Airship Dock</t>
   </si>
   <si>
-    <t>Government</t>
-  </si>
-  <si>
     <t>Military</t>
   </si>
   <si>
@@ -64,6 +49,36 @@
   </si>
   <si>
     <t>ResourceDepot</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>Vanderbilt</t>
+  </si>
+  <si>
+    <t>DistrictType</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Limit</t>
   </si>
 </sst>
 </file>
@@ -385,121 +400,133 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.54296875" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="1"/>
+      <c r="C9" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="1"/>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
+    <row r="11" spans="1:5" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>